<commit_message>
Mensajes entrevista Carlos: version final en el archivo oficial, eliminado el auxiliar
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/CFO/MENSAJES_ENTREVISTA_CARLOS.xlsx
+++ b/recursos/comercial/CFO/MENSAJES_ENTREVISTA_CARLOS.xlsx
@@ -464,7 +464,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VERSIÓN PRINCIPAL (se personaliza el nombre y, si aplica, una línea sobre su negocio):</t>
+          <t>VERSIÓN FINAL (aprobada 23/09) — se personaliza el nombre:</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Hola [NOMBRE], ¿cómo vas? Te escribo porque me acordé de ti viendo una entrevista. ¿Te acuerdas de Sandra, la que estaba en el equipo de Margarita? Se independizó y está haciendo entrevistas con expertos para empresarios. Acaba de sacar una con un financiero, Carlos Remolina, sobre algo en lo que ninguno de nosotros piensa: uno arma su equipo con contador y abogado, pero nunca con alguien que lea los números.</t>
+          <t>Hola [Nombre], ¿cómo estás? Te comparto una entrevista que le hizo Sandra Vega, la que estaba en el equipo de Margarita, a Carlos Remolina, financiero y mi socio de negocios. 🙌</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Hay un caso de un grupo de carwash en la Florida que me dejó fría: siete puntos vendiendo, y la solución fue cerrar tres porque entre más vendían más perdían. Y lo de que a veces uno pide crédito cuando no lo necesita.</t>
+          <t>¿Sabías que un negocio puede vender más y aun así perder más plata? Carlos cuenta el caso real de una cadena en Florida donde pasaba justo eso, y cómo lo resolvieron. También habla de por qué no siempre necesitas un crédito para crecer, y de las decisiones que tomamos por intuición cuando deberíamos mirar los números.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Te la dejo por si te sirve para tu negocio: [LINK]. Dura 45 minutos, pero se puede oír mientras uno hace otra cosa. Si la ves, cuéntame qué te pareció.</t>
+          <t>[link]</t>
         </is>
       </c>
     </row>
@@ -502,14 +502,14 @@
       <c r="A8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Te invito a verla y a compartirla con quien le pueda servir. Y si quieres que revisemos cómo están los números de tu negocio, escríbeme y lo vemos juntos. 😊</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>VERSIÓN CORTA (para los menos cercanos):</t>
-        </is>
-      </c>
+      <c r="A10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr"/>
@@ -517,50 +517,46 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Hola [NOMBRE], ¿cómo estás? Sandra, la que trabajaba con Margarita, ahora hace entrevistas para empresarios y acaba de sacar una con un financiero que me pareció muy buena: sobre por qué uno tiene contador y abogado pero nadie que le lea los números, y cuándo NO pedir crédito. Te la dejo por si te sirve: [LINK]. Un abrazo.</t>
+          <t>NOTAS DE ENVÍO:</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr"/>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>· Uno por uno, nunca por el grupo. Cambiar el nombre y, si hay confianza, una línea sobre su negocio.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr"/>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>· No más de 20 o 25 al día, para poder responder a quien conteste.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>NOTAS DE ENVÍO:</t>
+          <t>· Antes del primer envío, acordar con Carlos el paso siguiente: si alguien dice "sí, quiero", Diana le escribe a Carlos "te presento a [nombre], del grupo, quiere revisar sus números" y él lo contacta el mismo día.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>· Uno por uno, nunca por el grupo. Cambiar el nombre y, si hay confianza, agregar una línea sobre su negocio ("con lo del restaurante esto te puede servir").</t>
+          <t>· Nunca decir "socio en la empresa": la única empresa que el grupo conoce es Heiiu.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>· No más de 20 o 25 al día, para que no parezca campaña y para poder responder a quien conteste.</t>
-        </is>
-      </c>
+      <c r="A17" s="1" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>· Si alguien pregunta cómo contactar a Carlos: el WhatsApp está en la descripción del video. No dar el número directo en el mensaje inicial: que la entrevista lo venda.</t>
-        </is>
-      </c>
+      <c r="A18" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>· Si alguien pregunta si lo conoces: la verdad, sin más detalle del necesario: "sí, lo conozco y por eso sé que sabe de lo que habla".</t>
-        </is>
-      </c>
+      <c r="A19" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensaje entrevista Carlos: version final con landing ceremolina.com + WhatsApp directo, frase del podcast y calendario de envio
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/CFO/MENSAJES_ENTREVISTA_CARLOS.xlsx
+++ b/recursos/comercial/CFO/MENSAJES_ENTREVISTA_CARLOS.xlsx
@@ -464,7 +464,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VERSIÓN FINAL (aprobada 23/09) — se personaliza el nombre:</t>
+          <t>VERSIÓN FINAL (23/09) — se personaliza el nombre y se pega el link del video:</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>[link]</t>
+          <t>[link del video]</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Te invito a verla y a compartirla con quien le pueda servir. Y si quieres que revisemos cómo están los números de tu negocio, escríbeme y lo vemos juntos. 😊</t>
+          <t>Dura 45 minutos, pero se puede oír como un podcast mientras haces otra cosa.</t>
         </is>
       </c>
     </row>
@@ -512,51 +512,59 @@
       <c r="A10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Te invito a verla y a compartirla con quien le pueda servir. Y si quieres que revisemos cómo están los números de tu negocio, aquí está toda la información: ceremolina.com — o escríbele directo y dile que vas de mi parte: wa.me/573102748487 😊</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>NOTAS DE ENVÍO:</t>
-        </is>
-      </c>
+      <c r="A12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>· Uno por uno, nunca por el grupo. Cambiar el nombre y, si hay confianza, una línea sobre su negocio.</t>
-        </is>
-      </c>
+      <c r="A13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>· No más de 20 o 25 al día, para poder responder a quien conteste.</t>
+          <t>NOTAS DE ENVÍO:</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>· Antes del primer envío, acordar con Carlos el paso siguiente: si alguien dice "sí, quiero", Diana le escribe a Carlos "te presento a [nombre], del grupo, quiere revisar sus números" y él lo contacta el mismo día.</t>
+          <t>· Uno por uno, nunca por el grupo. Cambiar el nombre y, si hay confianza, una línea sobre su negocio.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
+          <t>· Hoy miércoles a las 8 PM los 20-25 cercanos; el domingo entre 5 y 8 PM el resto; después entre semana a las 8 PM. No más de 20-25 por día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>· Antes del primer envío, confirmar con Carlos: que ceremolina.com abre, que el Calendly está conectado a su calendario real, y que puede responder en menos de 48 horas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>· Probar el link wa.me desde el celular antes de enviar el primero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
           <t>· Nunca decir "socio en la empresa": la única empresa que el grupo conoce es Heiiu.</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensaje entrevista Carlos: notas con el grupo de tres para quien responde, regla de espectadora y confirmacion del cupo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/CFO/MENSAJES_ENTREVISTA_CARLOS.xlsx
+++ b/recursos/comercial/CFO/MENSAJES_ENTREVISTA_CARLOS.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -566,6 +566,27 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>· SI ALGUIEN RESPONDE "ME INTERESA": no mandarlo al link. Crear un grupo de WhatsApp de tres (Diana, Carlos y la persona) con este mensaje: "Carlos, te presento a [nombre], del grupo de Margarita. Tiene [negocio] y quiere revisar [lo que le duele]. Los dejo en buenas manos."</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>· Después de la presentación, Diana no vuelve a escribir en el grupo: la conversación es de Carlos y el cliente. Si Diana responde, el cliente le sigue escribiendo a ella y en dos semanas hay 20 grupos que dependen de ella. Presentar y quedarse de espectadora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>· Confirmar con Carlos que el cupo de 5 empresas al mes sigue vigente, para que la página y el mensaje digan lo mismo.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>